<commit_message>
feat: compare formulas. Prevent input overwrite.
- Add a `Difference Sheet` summary column, test dependencies, and regression tests for comparison accuracy and safe report publication.

- Preserve literal missing-value strings and compare formula expressions directly from the open workbooks.
- Apply whitespace normalization consistently and allocate unique report sheet names after truncation.
- Validate sheet selections and report missing inputs with resolved paths and working-directory guidance.
- Close workbook and writer resources on failure and replace reports only after a successful temporary-file save.
- Keep bold, centered, thin-bordered COMPARISON headers.

- Reject output paths that alias either input and write formula-like report values as literal text.
</commit_message>
<xml_diff>
--- a/example/a.xlsx
+++ b/example/a.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rejth\Downloads\ad_ucto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Dropbox\Work\godsdev-github\xlsx-compare\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{392ADDEC-0644-4F63-BF8D-7F5FF5A642DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0FB55D1-5B0D-4C45-8C48-58EE9E2453E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{42AC03BA-AE0B-4E1D-9B7A-ED345BAA2529}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="7740" xr2:uid="{42AC03BA-AE0B-4E1D-9B7A-ED345BAA2529}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B24A46B-7D43-4E69-A062-F3DAD8326EA5}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -417,6 +417,16 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <f>1+1</f>
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <f>1+2</f>
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: compare cells where a different formula have a different/same result
</commit_message>
<xml_diff>
--- a/example/a.xlsx
+++ b/example/a.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Dropbox\Work\godsdev-github\xlsx-compare\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0FB55D1-5B0D-4C45-8C48-58EE9E2453E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B075D173-5031-453A-B7FC-4EE3B86E66AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="7740" xr2:uid="{42AC03BA-AE0B-4E1D-9B7A-ED345BAA2529}"/>
   </bookViews>
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B24A46B-7D43-4E69-A062-F3DAD8326EA5}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -427,6 +427,12 @@
         <v>3</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <f>1+1</f>
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>